<commit_message>
Created generate client script
</commit_message>
<xml_diff>
--- a/projects/client-operations-dashboard/workbook/Client Operations Dashboard.xlsx
+++ b/projects/client-operations-dashboard/workbook/Client Operations Dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coult\Documents\GitHub\business-analytics-portfolio\projects\client-operations-dashboard\workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122F6044-399A-4905-857D-7C4726F63F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C047C7A-CEA2-4E6E-B252-94D8A3557ED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15585" yWindow="0" windowWidth="13320" windowHeight="15585" firstSheet="1" activeTab="3" xr2:uid="{F2C047C7-8673-4667-AD95-E88CE84B20A4}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="3" xr2:uid="{F2C047C7-8673-4667-AD95-E88CE84B20A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -24,10 +24,21 @@
     <sheet name="Inactive Queue" sheetId="9" r:id="rId9"/>
     <sheet name="Data Quality" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -371,9 +382,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -411,7 +422,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -517,7 +528,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -659,7 +670,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -692,7 +703,7 @@
     <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -703,7 +714,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="75">
+    <row r="2" spans="1:3" ht="45">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -715,7 +726,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="75">
+    <row r="3" spans="1:3" ht="45">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -726,7 +737,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="75">
+    <row r="4" spans="1:3" ht="45">
       <c r="A4" s="4" t="s">
         <v>8</v>
       </c>
@@ -737,7 +748,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="75">
+    <row r="5" spans="1:3" ht="45">
       <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
@@ -748,7 +759,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="75">
+    <row r="6" spans="1:3" ht="45">
       <c r="A6" s="4" t="s">
         <v>12</v>
       </c>
@@ -759,7 +770,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="90">
+    <row r="7" spans="1:3" ht="45">
       <c r="A7" s="4" t="s">
         <v>14</v>
       </c>

</xml_diff>